<commit_message>
fix: cleanup App.jsx and add jsconfig
</commit_message>
<xml_diff>
--- a/src/BACKUP/DER OPS NEW CRM 2021 (Only commo).xlsx
+++ b/src/BACKUP/DER OPS NEW CRM 2021 (Only commo).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omimr\mon-crm\src\BACKUP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54589B78-0450-47CF-AA07-F89A07F321BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF191F7-75F4-4F01-80FD-DD2150E0A62C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{64E2C1B3-2214-4A1F-A25C-111421665D0E}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64E2C1B3-2214-4A1F-A25C-111421665D0E}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4566" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4570" uniqueCount="164">
   <si>
     <t>ref</t>
   </si>
@@ -529,6 +529,9 @@
   <si>
     <t>CTR21007-corn-262.100000</t>
   </si>
+  <si>
+    <t>C4359</t>
+  </si>
 </sst>
 </file>
 
@@ -3303,8 +3306,8 @@
       <c r="M50" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="N50" s="2">
-        <v>4359</v>
+      <c r="N50" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="O50" s="2" t="s">
         <v>42</v>
@@ -3509,8 +3512,8 @@
       <c r="M54" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="N54" s="2">
-        <v>4359</v>
+      <c r="N54" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="O54" s="2" t="s">
         <v>42</v>
@@ -4486,8 +4489,8 @@
       <c r="M73" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="N73" s="2">
-        <v>4359</v>
+      <c r="N73" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="O73" s="2" t="s">
         <v>42</v>
@@ -4533,8 +4536,8 @@
       <c r="M74" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="N74" s="2">
-        <v>4359</v>
+      <c r="N74" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="O74" s="2" t="s">
         <v>42</v>

</xml_diff>